<commit_message>
doc/Flight.xlsx 引脚表补 LED(PG7) 与 W25Q64 六脚 (对齐接口配置表)
</commit_message>
<xml_diff>
--- a/doc/Flight.xlsx
+++ b/doc/Flight.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STM32Project\Flight\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\26718\OneDrive\桌面\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACB215E-E506-47DA-AF8A-E8179F655C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F600C77-E372-4C52-A754-44D53F95DA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="139">
   <si>
     <t>GND</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -507,6 +507,40 @@
   </si>
   <si>
     <t>I2C4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>PG7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flash W25Q64</t>
+  </si>
+  <si>
+    <t>PG6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF8</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -917,10 +951,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="10.53125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
@@ -1182,6 +1217,78 @@
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A30" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A32" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A33" s="5"/>
+      <c r="B33" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
UM982 迁移 UART4: USART2(PA2/PA3)→UART4(PA0/PA1) + 1PPS TIM2_CH1(PA0)→TIM2_CH3(PA2), DMA1_Stream2 复用
</commit_message>
<xml_diff>
--- a/doc/Flight.xlsx
+++ b/doc/Flight.xlsx
@@ -1,546 +1,449 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\26718\OneDrive\桌面\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STM32Project\Flight\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F600C77-E372-4C52-A754-44D53F95DA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B3DB91-6CA7-45B0-B66A-FE025A271F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="引脚" sheetId="1" r:id="rId1"/>
     <sheet name="接口配置" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="139">
-  <si>
-    <t>GND</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VCC</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CLK</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="136">
+  <si>
+    <t>设备</t>
+  </si>
+  <si>
+    <t>Buard Rate</t>
+  </si>
+  <si>
+    <t>采样频率</t>
+  </si>
+  <si>
+    <t>传感器引脚</t>
+  </si>
+  <si>
+    <t>STM32H723ZGT6引脚</t>
+  </si>
+  <si>
+    <t>STM32外设</t>
+  </si>
+  <si>
+    <t>DMA资源</t>
+  </si>
+  <si>
+    <t>中断优先级</t>
+  </si>
+  <si>
+    <t>功能说明</t>
+  </si>
+  <si>
+    <t>ADIS16505 IMU（SPI1 Burst）</t>
+  </si>
+  <si>
+    <t>954.861kHz</t>
+  </si>
+  <si>
+    <t>1000Hz</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>PC4</t>
+  </si>
+  <si>
+    <t>GPIO Output</t>
+  </si>
+  <si>
+    <t>SPI片选（软件控制）</t>
+  </si>
+  <si>
+    <t>SCLK</t>
+  </si>
+  <si>
+    <t>PA5</t>
+  </si>
+  <si>
+    <t>SPI1_SCK</t>
+  </si>
+  <si>
+    <t>SPI时钟</t>
+  </si>
+  <si>
+    <t>DOUT</t>
+  </si>
+  <si>
+    <t>PA6</t>
+  </si>
+  <si>
+    <t>SPI1_MISO</t>
+  </si>
+  <si>
+    <t>DMA1_Stream0</t>
+  </si>
+  <si>
+    <t>IMU数据输出</t>
   </si>
   <si>
     <t>DIN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DOUT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PA7</t>
+  </si>
+  <si>
+    <t>SPI1_MOSI</t>
+  </si>
+  <si>
+    <t>DMA1_Stream1</t>
+  </si>
+  <si>
+    <t>IMU数据输入</t>
+  </si>
+  <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>PA4</t>
+  </si>
+  <si>
+    <t>EXTI</t>
+  </si>
+  <si>
+    <t>数据就绪中断</t>
   </si>
   <si>
     <t>RESET</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC5</t>
+  </si>
+  <si>
+    <t>UM982 RTK GNSS</t>
+  </si>
+  <si>
+    <t>460800 Hz</t>
+  </si>
+  <si>
+    <t>10Hz</t>
+  </si>
+  <si>
+    <t>TXD</t>
+  </si>
+  <si>
+    <t>PA1</t>
+  </si>
+  <si>
+    <t>UART4_RX</t>
+  </si>
+  <si>
+    <t>DMA1 UART4_RX Circular</t>
+  </si>
+  <si>
+    <t>GNSS发送数据给STM32</t>
+  </si>
+  <si>
+    <t>RXD</t>
+  </si>
+  <si>
+    <t>PA0</t>
+  </si>
+  <si>
+    <t>UART4_TX</t>
+  </si>
+  <si>
+    <t>STM32发送配置命令</t>
   </si>
   <si>
     <t>PPS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADIS16505</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SPI1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA6</t>
-  </si>
-  <si>
-    <t>PA6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA3</t>
-  </si>
-  <si>
-    <t>PA3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CS</t>
-  </si>
-  <si>
-    <t>DOUT</t>
-  </si>
-  <si>
-    <t>PA5</t>
-  </si>
-  <si>
-    <t>DIN</t>
-  </si>
-  <si>
-    <t>PA7</t>
-  </si>
-  <si>
-    <t>UM982</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RX2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TX2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PPS</t>
-  </si>
-  <si>
-    <t>RST</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>PA2</t>
   </si>
   <si>
-    <t>PA2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PC4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA0</t>
-  </si>
-  <si>
-    <t>PA0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BMM350</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>TIM2_CH3</t>
+  </si>
+  <si>
+    <t>1PPS时间同步,使用定时器进行捕捉</t>
+  </si>
+  <si>
+    <t>BMM350 磁力计</t>
+  </si>
+  <si>
+    <t>400kHz</t>
+  </si>
+  <si>
+    <t>100Hz</t>
   </si>
   <si>
     <t>SCL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF14</t>
+  </si>
+  <si>
+    <t>I2C4_SCL</t>
+  </si>
+  <si>
+    <t>I2C时钟</t>
   </si>
   <si>
     <t>SDA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF15</t>
+  </si>
+  <si>
+    <t>I2C4_SDA</t>
+  </si>
+  <si>
+    <t>I2C数据</t>
   </si>
   <si>
     <t>INT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USART2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>设备</t>
-  </si>
-  <si>
-    <t>传感器引脚</t>
-  </si>
-  <si>
-    <t>STM32H723ZGT6引脚</t>
-  </si>
-  <si>
-    <t>STM32外设</t>
-  </si>
-  <si>
-    <t>功能说明</t>
-  </si>
-  <si>
-    <t>GPIO Output</t>
-  </si>
-  <si>
-    <t>SPI片选（软件控制）</t>
-  </si>
-  <si>
-    <t>SCLK</t>
-  </si>
-  <si>
-    <t>SPI1_SCK</t>
-  </si>
-  <si>
-    <t>SPI时钟</t>
-  </si>
-  <si>
-    <t>SPI1_MISO</t>
-  </si>
-  <si>
-    <t>IMU数据输出</t>
-  </si>
-  <si>
-    <t>SPI1_MOSI</t>
-  </si>
-  <si>
-    <t>IMU数据输入</t>
-  </si>
-  <si>
-    <t>数据就绪中断</t>
-  </si>
-  <si>
-    <t>气压数据中断</t>
-  </si>
-  <si>
-    <t>BMM350 磁力计</t>
-  </si>
-  <si>
-    <t>I2C时钟</t>
-  </si>
-  <si>
-    <t>I2C数据</t>
+  </si>
+  <si>
+    <t>PF12</t>
+  </si>
+  <si>
+    <t>EXTI12</t>
   </si>
   <si>
     <t>磁场数据中断</t>
   </si>
   <si>
-    <t>UM982 RTK GNSS</t>
-  </si>
-  <si>
-    <t>TXD</t>
-  </si>
-  <si>
-    <t>USART2_RX</t>
-  </si>
-  <si>
-    <t>GNSS发送数据给STM32</t>
-  </si>
-  <si>
-    <t>RXD</t>
-  </si>
-  <si>
-    <t>STM32发送配置命令</t>
-  </si>
-  <si>
-    <t>TIM2_CH1</t>
-  </si>
-  <si>
-    <t>DMA资源</t>
-  </si>
-  <si>
-    <t>中断优先级</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EXTI</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1PPS时间同步,使用定时器进行捕捉</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USART2_TX</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADIS16505 IMU（SPI1 Burst）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>954.861kHz</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Buard Rate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>采样频率</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1000Hz</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>100Hz</t>
-  </si>
-  <si>
-    <t>LED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PG7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>调试串口</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DMA1_Stream3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DMA1_Stream4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DMA1_Stream1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DMA1_Stream0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>调试</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USART1_TX</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USART1_RX</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BMP585</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>BMP585 气压计</t>
   </si>
   <si>
     <t>PB10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I2C2_SCL</t>
   </si>
   <si>
     <t>PB11</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PE13</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I2C2_SDA</t>
   </si>
   <si>
     <t>DMA2 Stream0 → I2C2_RX
 DMA2 Stream1 → I2C2_TX</t>
+  </si>
+  <si>
+    <t>PE13</t>
+  </si>
+  <si>
+    <t>EXTI13</t>
+  </si>
+  <si>
+    <t>气压数据中断</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>PG7</t>
+  </si>
+  <si>
+    <t>调试串口</t>
+  </si>
+  <si>
+    <t>PA9</t>
+  </si>
+  <si>
+    <t>USART1_TX</t>
+  </si>
+  <si>
+    <t>DMA1_Stream4</t>
+  </si>
+  <si>
+    <t>调试</t>
+  </si>
+  <si>
+    <t>PA10</t>
+  </si>
+  <si>
+    <t>USART1_RX</t>
+  </si>
+  <si>
+    <t>DMA1_Stream3</t>
+  </si>
+  <si>
+    <t>Flash W25Q64</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_NCS-PG6</t>
+  </si>
+  <si>
+    <t>DO</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_IO1-PF9</t>
+  </si>
+  <si>
+    <t>WP(IO2)</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_IO2-PF7</t>
+  </si>
+  <si>
+    <t>HOLD(IO3)</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_IO3-PF6</t>
+  </si>
+  <si>
+    <t>CLK</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_CLK-PF10</t>
+  </si>
+  <si>
+    <t>DI(IO0)</t>
+  </si>
+  <si>
+    <t>OCTOSPIM_P1_IO0-PF8</t>
+  </si>
+  <si>
+    <t>ADIS16505</t>
+  </si>
+  <si>
+    <t>SPI1</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>UM982</t>
+  </si>
+  <si>
+    <t>UART4</t>
+  </si>
+  <si>
+    <t>RX2</t>
+  </si>
+  <si>
+    <t>TX2</t>
+  </si>
+  <si>
+    <t>RST</t>
+  </si>
+  <si>
+    <t>PC1</t>
+  </si>
+  <si>
+    <t>BMM350</t>
+  </si>
+  <si>
+    <t>I2C4</t>
+  </si>
+  <si>
+    <t>BMP585</t>
+  </si>
+  <si>
+    <t>I2C2</t>
+  </si>
+  <si>
+    <t>PG6</t>
+  </si>
+  <si>
+    <t>PF9</t>
+  </si>
+  <si>
+    <t>PF7</t>
+  </si>
+  <si>
+    <t>PF6</t>
+  </si>
+  <si>
+    <t>PF10</t>
+  </si>
+  <si>
+    <t>PF8</t>
+  </si>
+  <si>
+    <t>miniTF</t>
+  </si>
+  <si>
+    <t>SDMMC1_D0_PC8</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>EXTI13</t>
+    <t>SDMMC1_D1_PC9</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>DMA1 USART2_RX Circular</t>
+    <t>SDMMC1_D2_PC10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PC5</t>
+    <t>SDMMC1_D3_PC11</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>100Hz</t>
+    <t>SDMMC1_CMD_PD2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>400kHz</t>
+    <t>SDMMC1_CK_PC12</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>10Hz</t>
+    <t>DATA0</t>
+  </si>
+  <si>
+    <t>DATA1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>BMP585 气压计</t>
+    <t>DATA2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Flash W25Q64</t>
+    <t>CMD</t>
+  </si>
+  <si>
+    <t>DATA3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CS</t>
+    <t>PC8</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>DO</t>
+    <t>PC9</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>WP(IO2)</t>
+    <t>PC10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>HOLD(IO3)</t>
+    <t>PC11</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CLK</t>
+    <t>PD2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>DI(IO0)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_IO2-PF7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_IO1-PF9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_NCS-PG6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_IO3-PF6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_CLK-PF10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OCTOSPIM_P1_IO0-PF8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>460800 Hz</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C2_SDA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C2_SCL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF14</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SCL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SDA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>INT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF12</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C4_SCL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C4_SDA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EXTI12</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>LED</t>
-  </si>
-  <si>
-    <t>PG7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Flash W25Q64</t>
-  </si>
-  <si>
-    <t>PG6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PF8</t>
+    <t>PC12</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -642,7 +545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -671,6 +574,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -951,7 +857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13.265625" bestFit="1" customWidth="1"/>
@@ -960,45 +866,45 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5" t="s">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="D5" s="5"/>
     </row>
@@ -1010,55 +916,55 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="5" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="12" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="13" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="13" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="5" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1078,50 +984,50 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="5" t="s">
-        <v>22</v>
+        <v>102</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>37</v>
+        <v>103</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="5" t="s">
-        <v>23</v>
+        <v>104</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="5" t="s">
-        <v>24</v>
+        <v>105</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="12" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="5" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>29</v>
+        <v>107</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -1134,40 +1040,40 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="5" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>129</v>
+        <v>109</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="5" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>120</v>
+        <v>56</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="5" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>121</v>
+        <v>60</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="5" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>125</v>
+        <v>64</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -1180,40 +1086,40 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="5" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="5" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="5" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="5" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -1226,10 +1132,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="5" t="s">
-        <v>130</v>
+        <v>76</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>131</v>
+        <v>77</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -1242,10 +1148,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="5" t="s">
-        <v>132</v>
+        <v>86</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -1253,7 +1159,7 @@
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -1261,7 +1167,7 @@
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
@@ -1269,7 +1175,7 @@
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
@@ -1277,7 +1183,7 @@
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -1285,10 +1191,66 @@
     <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A39" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A43" s="5"/>
+      <c r="B43" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1297,8 +1259,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2FD369E-E8D4-4915-8284-0825775DBC68}">
-  <dimension ref="A1:AB31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:AB34"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1313,31 +1275,31 @@
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
@@ -1359,29 +1321,29 @@
       <c r="AA1" s="5"/>
       <c r="AB1" s="5"/>
     </row>
-    <row r="2" spans="1:28" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:28" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
       <c r="I2" s="7" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
@@ -1408,18 +1370,18 @@
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="8"/>
       <c r="I3" s="7" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -1446,22 +1408,22 @@
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="H4" s="8">
         <v>3</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
@@ -1488,22 +1450,22 @@
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="H5" s="8">
         <v>3</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
@@ -1530,20 +1492,20 @@
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7" t="s">
-        <v>88</v>
+        <v>30</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="8">
         <v>2</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
@@ -1570,10 +1532,10 @@
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -1601,31 +1563,31 @@
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>37</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>102</v>
+        <v>38</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="H8" s="8">
         <v>3</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
@@ -1652,19 +1614,19 @@
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="H9" s="8">
         <v>5</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
@@ -1691,20 +1653,20 @@
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="8">
         <v>1</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
@@ -1727,29 +1689,19 @@
       <c r="AB10" s="5"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A11" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" t="s">
-        <v>101</v>
-      </c>
-      <c r="C11" t="s">
-        <v>75</v>
-      </c>
+      <c r="A11" s="7"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
       <c r="D11" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>126</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="8"/>
-      <c r="I11" s="7" t="s">
-        <v>55</v>
-      </c>
+      <c r="I11" s="7"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
@@ -1771,22 +1723,28 @@
       <c r="AB11" s="5"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
+      <c r="A12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
       <c r="D12" s="7" t="s">
-        <v>123</v>
+        <v>55</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>127</v>
+        <v>57</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="8"/>
       <c r="I12" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
@@ -1813,20 +1771,18 @@
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>128</v>
+        <v>61</v>
       </c>
       <c r="G13" s="7"/>
-      <c r="H13" s="8">
-        <v>7</v>
-      </c>
+      <c r="H13" s="8"/>
       <c r="I13" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
@@ -1849,27 +1805,25 @@
       <c r="AB13" s="5"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A14" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>92</v>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>64</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>119</v>
+        <v>65</v>
       </c>
       <c r="G14" s="7"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="7"/>
+      <c r="H14" s="8">
+        <v>7</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -1890,22 +1844,26 @@
       <c r="AA14" s="5"/>
       <c r="AB14" s="5"/>
     </row>
-    <row r="15" spans="1:28" ht="27.75" x14ac:dyDescent="0.4">
-      <c r="A15" s="7"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="7"/>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.4">
+      <c r="A15" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>54</v>
+      </c>
       <c r="D15" s="5" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="G15" s="7"/>
       <c r="H15" s="8"/>
       <c r="I15" s="7"/>
       <c r="J15" s="5"/>
@@ -1928,26 +1886,24 @@
       <c r="AA15" s="5"/>
       <c r="AB15" s="5"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:28" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="7"/>
       <c r="B16" s="11"/>
       <c r="C16" s="7"/>
       <c r="D16" s="5" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="G16" s="7"/>
-      <c r="H16" s="8">
-        <v>7</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>53</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="8"/>
+      <c r="I16" s="7"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
@@ -1969,19 +1925,25 @@
       <c r="AB16" s="5"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A17" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" s="7"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>74</v>
+      </c>
       <c r="G17" s="7"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="7"/>
+      <c r="H17" s="8">
+        <v>7</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>75</v>
+      </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
@@ -2003,27 +1965,19 @@
       <c r="AB17" s="5"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A18" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
+      <c r="A18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="H18" s="8">
-        <v>5</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>85</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="7"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
@@ -2045,7 +1999,9 @@
       <c r="AB18" s="5"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A19" s="7"/>
+      <c r="A19" s="7" t="s">
+        <v>78</v>
+      </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -2053,7 +2009,7 @@
         <v>79</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>81</v>
@@ -2062,7 +2018,7 @@
         <v>5</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
@@ -2089,11 +2045,21 @@
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
+      <c r="E20" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" s="8">
+        <v>5</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>82</v>
+      </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
@@ -2115,17 +2081,11 @@
       <c r="AB20" s="5"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A21" s="7" t="s">
-        <v>104</v>
-      </c>
+      <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
-      <c r="D21" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>113</v>
-      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
@@ -2151,14 +2111,16 @@
       <c r="AB21" s="5"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A22" s="7"/>
+      <c r="A22" s="7" t="s">
+        <v>86</v>
+      </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7" t="s">
-        <v>106</v>
+        <v>12</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -2189,15 +2151,15 @@
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="5"/>
+      <c r="I23" s="7"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
@@ -2223,10 +2185,10 @@
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E24" t="s">
-        <v>114</v>
+        <v>90</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>91</v>
       </c>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
@@ -2257,10 +2219,10 @@
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>115</v>
+        <v>92</v>
+      </c>
+      <c r="E25" t="s">
+        <v>93</v>
       </c>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
@@ -2291,10 +2253,10 @@
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
@@ -2324,8 +2286,12 @@
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
+      <c r="D27" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>97</v>
+      </c>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
@@ -2381,25 +2347,89 @@
       <c r="AB28" s="5"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
+      <c r="A29" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" t="s">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>119</v>
+      </c>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
+      <c r="V29" s="5"/>
+      <c r="W29" s="5"/>
+      <c r="X29" s="5"/>
+      <c r="Y29" s="5"/>
+      <c r="Z29" s="5"/>
+      <c r="AA29" s="5"/>
+      <c r="AB29" s="5"/>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
+      <c r="D31" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" t="s">
+        <v>129</v>
+      </c>
+      <c r="E32" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D33" t="s">
+        <v>128</v>
+      </c>
+      <c r="E33" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D34" t="s">
+        <v>94</v>
+      </c>
+      <c r="E34" t="s">
+        <v>124</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>